<commit_message>
Chart: only the UGX creditor is typed Payable, so the import goes through
At the end of the import ERPNext makes the first Payable ledger it finds
the company's default payable account and saves the company, which
refuses one not in the company currency ("Default Payable Account
currency must be same as company's default currency"); the whole import
is then undone. The client's chart had three Payable ledgers, two of them
in GBP and USD.

22010102 (GBP) and 22010104 (USD) are now left without the Payable type;
set it on them after the import if suppliers will be billed in those
currencies. coa_changes.txt says so.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo_import/00_chart_of_accounts.xlsx
+++ b/demo_import/00_chart_of_accounts.xlsx
@@ -4267,11 +4267,7 @@
       <c r="E129" t="n">
         <v>0</v>
       </c>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>Payable</t>
-        </is>
-      </c>
+      <c r="F129" t="inlineStr"/>
       <c r="G129" t="inlineStr"/>
       <c r="H129" t="inlineStr">
         <is>
@@ -4331,11 +4327,7 @@
       <c r="E131" t="n">
         <v>0</v>
       </c>
-      <c r="F131" t="inlineStr">
-        <is>
-          <t>Payable</t>
-        </is>
-      </c>
+      <c r="F131" t="inlineStr"/>
       <c r="G131" t="inlineStr"/>
       <c r="H131" t="inlineStr">
         <is>

</xml_diff>